<commit_message>
got the new data formatting working; now I only need to add the curve filter and then colours and then we're so back
</commit_message>
<xml_diff>
--- a/proliferation_growth_curves/Incucyte_sheets/processed/r1_processed.xlsx
+++ b/proliferation_growth_curves/Incucyte_sheets/processed/r1_processed.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,7 +592,7 @@
         <v>23.78014125</v>
       </c>
       <c r="K3" t="n">
-        <v>33.97371124999999</v>
+        <v>33.97371125</v>
       </c>
       <c r="L3" t="n">
         <v>14.791916625</v>
@@ -684,7 +684,7 @@
         <v>19.108665</v>
       </c>
       <c r="G5" t="n">
-        <v>39.675745</v>
+        <v>39.67574499999999</v>
       </c>
       <c r="H5" t="n">
         <v>16.42569625</v>
@@ -736,7 +736,7 @@
         <v>20.556685</v>
       </c>
       <c r="G6" t="n">
-        <v>45.249935</v>
+        <v>45.24993500000001</v>
       </c>
       <c r="H6" t="n">
         <v>16.94776375</v>
@@ -748,7 +748,7 @@
         <v>34.3008525</v>
       </c>
       <c r="K6" t="n">
-        <v>51.767805</v>
+        <v>51.76780500000001</v>
       </c>
       <c r="L6" t="n">
         <v>22.5531225</v>
@@ -794,7 +794,7 @@
         <v>20.11368625</v>
       </c>
       <c r="I7" t="n">
-        <v>45.95910500000001</v>
+        <v>45.959105</v>
       </c>
       <c r="J7" t="n">
         <v>40.732365</v>
@@ -812,10 +812,10 @@
         <v>50.17283500000001</v>
       </c>
       <c r="O7" t="n">
-        <v>44.3695175</v>
+        <v>44.36951749999999</v>
       </c>
       <c r="P7" t="n">
-        <v>42.68795249999999</v>
+        <v>42.6879525</v>
       </c>
     </row>
     <row r="8">
@@ -846,13 +846,13 @@
         <v>23.74723375</v>
       </c>
       <c r="I8" t="n">
-        <v>54.75184</v>
+        <v>54.75183999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>47.69957125000001</v>
+        <v>47.69957125</v>
       </c>
       <c r="K8" t="n">
-        <v>73.54741249999999</v>
+        <v>73.54741250000001</v>
       </c>
       <c r="L8" t="n">
         <v>31.2691475</v>
@@ -864,7 +864,7 @@
         <v>56.82566749999999</v>
       </c>
       <c r="O8" t="n">
-        <v>52.09189</v>
+        <v>52.09188999999999</v>
       </c>
       <c r="P8" t="n">
         <v>50.03530375</v>
@@ -901,7 +901,7 @@
         <v>65.659705</v>
       </c>
       <c r="J9" t="n">
-        <v>58.3349175</v>
+        <v>58.33491750000001</v>
       </c>
       <c r="K9" t="n">
         <v>84.4678475</v>
@@ -919,7 +919,7 @@
         <v>63.23652375</v>
       </c>
       <c r="P9" t="n">
-        <v>60.50221124999999</v>
+        <v>60.50221125</v>
       </c>
     </row>
     <row r="10">
@@ -941,7 +941,7 @@
         <v>44.80348125</v>
       </c>
       <c r="F10" t="n">
-        <v>37.57561125</v>
+        <v>37.57561124999999</v>
       </c>
       <c r="G10" t="n">
         <v>79.10964125</v>
@@ -953,7 +953,7 @@
         <v>74.71906625</v>
       </c>
       <c r="J10" t="n">
-        <v>67.55589624999999</v>
+        <v>67.55589625</v>
       </c>
       <c r="K10" t="n">
         <v>92.10002249999999</v>
@@ -965,10 +965,10 @@
         <v>35.7864225</v>
       </c>
       <c r="N10" t="n">
-        <v>73.73484375000001</v>
+        <v>73.73484375</v>
       </c>
       <c r="O10" t="n">
-        <v>72.09157375000001</v>
+        <v>72.09157374999999</v>
       </c>
       <c r="P10" t="n">
         <v>70.10812625</v>
@@ -1002,7 +1002,7 @@
         <v>35.84429875</v>
       </c>
       <c r="I11" t="n">
-        <v>81.31295249999999</v>
+        <v>81.31295250000001</v>
       </c>
       <c r="J11" t="n">
         <v>74.68695</v>
@@ -1011,7 +1011,7 @@
         <v>95.1623225</v>
       </c>
       <c r="L11" t="n">
-        <v>54.90393125</v>
+        <v>54.90393124999999</v>
       </c>
       <c r="M11" t="n">
         <v>38.12338625</v>
@@ -1023,7 +1023,7 @@
         <v>80.9795125</v>
       </c>
       <c r="P11" t="n">
-        <v>77.3049625</v>
+        <v>77.30496249999999</v>
       </c>
     </row>
     <row r="12">
@@ -1042,7 +1042,7 @@
         <v>44</v>
       </c>
       <c r="E12" t="n">
-        <v>54.725425</v>
+        <v>54.72542499999999</v>
       </c>
       <c r="F12" t="n">
         <v>43.62658125</v>
@@ -1054,28 +1054,28 @@
         <v>41.8484925</v>
       </c>
       <c r="I12" t="n">
-        <v>88.16239999999999</v>
+        <v>88.16240000000001</v>
       </c>
       <c r="J12" t="n">
         <v>83.10793125000001</v>
       </c>
       <c r="K12" t="n">
-        <v>97.02997125</v>
+        <v>97.02997124999999</v>
       </c>
       <c r="L12" t="n">
-        <v>63.0942125</v>
+        <v>63.09421249999999</v>
       </c>
       <c r="M12" t="n">
         <v>42.56467125</v>
       </c>
       <c r="N12" t="n">
-        <v>82.431465</v>
+        <v>82.43146499999999</v>
       </c>
       <c r="O12" t="n">
-        <v>87.20843500000001</v>
+        <v>87.20843499999999</v>
       </c>
       <c r="P12" t="n">
-        <v>85.47519750000001</v>
+        <v>85.47519749999999</v>
       </c>
     </row>
     <row r="13">
@@ -1094,25 +1094,25 @@
         <v>48</v>
       </c>
       <c r="E13" t="n">
-        <v>69.59625124999999</v>
+        <v>69.59625125000001</v>
       </c>
       <c r="F13" t="n">
         <v>65.0155575</v>
       </c>
       <c r="G13" t="n">
-        <v>96.18448875</v>
+        <v>96.18448874999999</v>
       </c>
       <c r="H13" t="n">
         <v>56.99643625</v>
       </c>
       <c r="I13" t="n">
-        <v>97.402355</v>
+        <v>97.40235500000001</v>
       </c>
       <c r="J13" t="n">
-        <v>95.31951874999999</v>
+        <v>95.31951875</v>
       </c>
       <c r="K13" t="n">
-        <v>99.68587375000001</v>
+        <v>99.68587374999998</v>
       </c>
       <c r="L13" t="n">
         <v>82.68072125</v>
@@ -1124,7 +1124,7 @@
         <v>95.46951375</v>
       </c>
       <c r="O13" t="n">
-        <v>97.23854375000001</v>
+        <v>97.23854374999999</v>
       </c>
       <c r="P13" t="n">
         <v>95.59627374999999</v>
@@ -1155,7 +1155,7 @@
         <v>94.81824</v>
       </c>
       <c r="H14" t="n">
-        <v>60.194635</v>
+        <v>60.19463500000001</v>
       </c>
       <c r="I14" t="n">
         <v>97.06249</v>
@@ -1164,10 +1164,10 @@
         <v>95.6463275</v>
       </c>
       <c r="K14" t="n">
-        <v>99.50287</v>
+        <v>99.50286999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>85.71844374999999</v>
+        <v>85.71844375000001</v>
       </c>
       <c r="M14" t="n">
         <v>58.12277125</v>
@@ -1198,7 +1198,7 @@
         <v>56</v>
       </c>
       <c r="E15" t="n">
-        <v>72.19913124999999</v>
+        <v>72.19913125000001</v>
       </c>
       <c r="F15" t="n">
         <v>63.085925</v>
@@ -1207,7 +1207,7 @@
         <v>94.18683625</v>
       </c>
       <c r="H15" t="n">
-        <v>63.9833475</v>
+        <v>63.98334750000001</v>
       </c>
       <c r="I15" t="n">
         <v>97.86777875</v>
@@ -1216,7 +1216,7 @@
         <v>97.17726999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>99.48083500000001</v>
+        <v>99.48083499999998</v>
       </c>
       <c r="L15" t="n">
         <v>90.00617625</v>
@@ -1225,13 +1225,13 @@
         <v>62.4800225</v>
       </c>
       <c r="N15" t="n">
-        <v>92.81031874999999</v>
+        <v>92.81031875000001</v>
       </c>
       <c r="O15" t="n">
-        <v>98.50023999999999</v>
+        <v>98.50024000000001</v>
       </c>
       <c r="P15" t="n">
-        <v>97.51360124999999</v>
+        <v>97.51360125000001</v>
       </c>
     </row>
     <row r="16">
@@ -1250,19 +1250,19 @@
         <v>60</v>
       </c>
       <c r="E16" t="n">
-        <v>74.20666625</v>
+        <v>74.20666624999998</v>
       </c>
       <c r="F16" t="n">
         <v>64.63278</v>
       </c>
       <c r="G16" t="n">
-        <v>94.46369</v>
+        <v>94.46368999999999</v>
       </c>
       <c r="H16" t="n">
         <v>70.9829775</v>
       </c>
       <c r="I16" t="n">
-        <v>98.24543249999999</v>
+        <v>98.24543250000001</v>
       </c>
       <c r="J16" t="n">
         <v>97.7821325</v>
@@ -1277,13 +1277,13 @@
         <v>65.7095925</v>
       </c>
       <c r="N16" t="n">
-        <v>93.10970624999999</v>
+        <v>93.10970625</v>
       </c>
       <c r="O16" t="n">
         <v>98.95161874999999</v>
       </c>
       <c r="P16" t="n">
-        <v>97.84124875000001</v>
+        <v>97.84124874999998</v>
       </c>
     </row>
     <row r="17">
@@ -1302,10 +1302,10 @@
         <v>64</v>
       </c>
       <c r="E17" t="n">
-        <v>78.54631999999999</v>
+        <v>78.54632000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>68.29519875</v>
+        <v>68.29519875000001</v>
       </c>
       <c r="G17" t="n">
         <v>94.92905875</v>
@@ -1314,16 +1314,16 @@
         <v>77.81173874999999</v>
       </c>
       <c r="I17" t="n">
-        <v>98.33709124999999</v>
+        <v>98.33709125</v>
       </c>
       <c r="J17" t="n">
-        <v>98.26449000000001</v>
+        <v>98.26449</v>
       </c>
       <c r="K17" t="n">
         <v>99.42542875000001</v>
       </c>
       <c r="L17" t="n">
-        <v>95.272595</v>
+        <v>95.27259500000001</v>
       </c>
       <c r="M17" t="n">
         <v>70.04543624999999</v>
@@ -1332,7 +1332,7 @@
         <v>93.03027750000001</v>
       </c>
       <c r="O17" t="n">
-        <v>99.09913874999999</v>
+        <v>99.09913875000001</v>
       </c>
       <c r="P17" t="n">
         <v>98.23297375</v>
@@ -1357,7 +1357,7 @@
         <v>80.42062250000001</v>
       </c>
       <c r="F18" t="n">
-        <v>69.54998499999999</v>
+        <v>69.54998500000001</v>
       </c>
       <c r="G18" t="n">
         <v>95.291855</v>
@@ -1381,10 +1381,10 @@
         <v>71.92412999999999</v>
       </c>
       <c r="N18" t="n">
-        <v>93.2787625</v>
+        <v>93.27876250000001</v>
       </c>
       <c r="O18" t="n">
-        <v>99.1499275</v>
+        <v>99.14992749999999</v>
       </c>
       <c r="P18" t="n">
         <v>98.48812624999999</v>
@@ -1412,7 +1412,7 @@
         <v>92.88213500000001</v>
       </c>
       <c r="G19" t="n">
-        <v>99.22212375000001</v>
+        <v>99.22212374999999</v>
       </c>
       <c r="H19" t="n">
         <v>95.13983875</v>
@@ -1436,323 +1436,11 @@
         <v>99.38851749999999</v>
       </c>
       <c r="O19" t="n">
-        <v>99.97472375000001</v>
+        <v>99.97472375</v>
       </c>
       <c r="P19" t="n">
         <v>99.94500500000001</v>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>slope</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>1.06719669627193</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>z.test</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>0.6413398636229423</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>1.039957804580897</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>stdev</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>0.1600116292400008</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>z.score</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>0.170230700233528</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>sem</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>0.05333720974666695</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>95 ci</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>1.144498735684364</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>q3</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>1.163392480263158</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>q1</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>0.8995343289473683</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>1.5*iqr</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>0.3957872269736841</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>-0.5037471019736842</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>1.559179707236842</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1765,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1976,7 +1664,7 @@
         <v>36.87299625</v>
       </c>
       <c r="H6" t="n">
-        <v>37.16046375</v>
+        <v>37.16046375000001</v>
       </c>
       <c r="I6" t="n">
         <v>31.524093125</v>
@@ -2044,13 +1732,13 @@
         <v>51.225705625</v>
       </c>
       <c r="H8" t="n">
-        <v>52.40827999999999</v>
+        <v>52.40828</v>
       </c>
       <c r="I8" t="n">
         <v>41.48614125</v>
       </c>
       <c r="J8" t="n">
-        <v>51.063596875</v>
+        <v>51.06359687499999</v>
       </c>
     </row>
     <row r="9">
@@ -2075,7 +1763,7 @@
         <v>50.00629375</v>
       </c>
       <c r="G9" t="n">
-        <v>61.99731125</v>
+        <v>61.99731125000001</v>
       </c>
       <c r="H9" t="n">
         <v>61.837673125</v>
@@ -2103,19 +1791,19 @@
         <v>36</v>
       </c>
       <c r="E10" t="n">
-        <v>41.18954625</v>
+        <v>41.18954624999999</v>
       </c>
       <c r="F10" t="n">
         <v>55.72781625</v>
       </c>
       <c r="G10" t="n">
-        <v>71.13748124999999</v>
+        <v>71.13748125000001</v>
       </c>
       <c r="H10" t="n">
         <v>69.80762874999999</v>
       </c>
       <c r="I10" t="n">
-        <v>54.76063312500001</v>
+        <v>54.760633125</v>
       </c>
       <c r="J10" t="n">
         <v>71.09985</v>
@@ -2143,13 +1831,13 @@
         <v>60.44432875</v>
       </c>
       <c r="G11" t="n">
-        <v>77.99995125</v>
+        <v>77.99995125000001</v>
       </c>
       <c r="H11" t="n">
         <v>75.03312687499999</v>
       </c>
       <c r="I11" t="n">
-        <v>57.2979925</v>
+        <v>57.29799250000001</v>
       </c>
       <c r="J11" t="n">
         <v>79.14223749999999</v>
@@ -2171,22 +1859,22 @@
         <v>44</v>
       </c>
       <c r="E12" t="n">
-        <v>49.176003125</v>
+        <v>49.17600312499999</v>
       </c>
       <c r="F12" t="n">
         <v>64.706754375</v>
       </c>
       <c r="G12" t="n">
-        <v>85.635165625</v>
+        <v>85.63516562500001</v>
       </c>
       <c r="H12" t="n">
         <v>80.06209187499999</v>
       </c>
       <c r="I12" t="n">
-        <v>62.498068125</v>
+        <v>62.49806812499999</v>
       </c>
       <c r="J12" t="n">
-        <v>86.34181625000001</v>
+        <v>86.34181624999999</v>
       </c>
     </row>
     <row r="13">
@@ -2205,16 +1893,16 @@
         <v>48</v>
       </c>
       <c r="E13" t="n">
-        <v>67.305904375</v>
+        <v>67.30590437500001</v>
       </c>
       <c r="F13" t="n">
-        <v>76.5904625</v>
+        <v>76.59046249999999</v>
       </c>
       <c r="G13" t="n">
-        <v>96.36093687499999</v>
+        <v>96.36093687500001</v>
       </c>
       <c r="H13" t="n">
-        <v>91.18329750000001</v>
+        <v>91.18329749999999</v>
       </c>
       <c r="I13" t="n">
         <v>78.01571250000001</v>
@@ -2282,13 +1970,13 @@
         <v>97.52252437499999</v>
       </c>
       <c r="H15" t="n">
-        <v>94.74350562500001</v>
+        <v>94.74350562499998</v>
       </c>
       <c r="I15" t="n">
-        <v>77.64517062499999</v>
+        <v>77.64517062500001</v>
       </c>
       <c r="J15" t="n">
-        <v>98.00692062499999</v>
+        <v>98.00692062500001</v>
       </c>
     </row>
     <row r="16">
@@ -2313,16 +2001,16 @@
         <v>82.72333374999999</v>
       </c>
       <c r="G16" t="n">
-        <v>98.01378249999999</v>
+        <v>98.0137825</v>
       </c>
       <c r="H16" t="n">
         <v>96.217314375</v>
       </c>
       <c r="I16" t="n">
-        <v>79.40964937499999</v>
+        <v>79.409649375</v>
       </c>
       <c r="J16" t="n">
-        <v>98.39643375</v>
+        <v>98.39643374999999</v>
       </c>
     </row>
     <row r="17">
@@ -2341,7 +2029,7 @@
         <v>64</v>
       </c>
       <c r="E17" t="n">
-        <v>73.42075937499999</v>
+        <v>73.42075937500002</v>
       </c>
       <c r="F17" t="n">
         <v>86.37039874999999</v>
@@ -2375,7 +2063,7 @@
         <v>68</v>
       </c>
       <c r="E18" t="n">
-        <v>74.98530375</v>
+        <v>74.98530375000001</v>
       </c>
       <c r="F18" t="n">
         <v>88.97380812500001</v>
@@ -2387,7 +2075,7 @@
         <v>97.785425</v>
       </c>
       <c r="I18" t="n">
-        <v>82.60144625</v>
+        <v>82.60144625000001</v>
       </c>
       <c r="J18" t="n">
         <v>98.81902687499999</v>
@@ -2424,248 +2112,8 @@
         <v>96.130793125</v>
       </c>
       <c r="J19" t="n">
-        <v>99.95986437500001</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>slope</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>1.06719669627193</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>z.test</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>0.6413398636229423</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>1.039957804580897</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>stdev</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>0.1600116292400008</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>z.score</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>0.170230700233528</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>sem</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>0.05333720974666695</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>95 ci</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>1.144498735684364</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>q3</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>1.163392480263158</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>q1</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>0.8995343289473683</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>1.5*iqr</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>0.3957872269736841</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>-0.5037471019736842</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>1.559179707236842</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+        <v>99.959864375</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>